<commit_message>
Update creative workbook immigration share
</commit_message>
<xml_diff>
--- a/data/exports/creative-post-video-slogan-stats.xlsx
+++ b/data/exports/creative-post-video-slogan-stats.xlsx
@@ -20,7 +20,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Video Type Summary'!$A$1:$L$6</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Overall Immigration Share'!$A$1:$G$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Overall Immigration Share'!$A$1:$K$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Creative Format Summary'!$A$1:$N$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Tag Overview Videos'!$A$1:$L$105</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Tag Overview All Posts'!$A$1:$L$156</definedName>
@@ -234,16 +234,20 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="OverallImmigrationShareTable" displayName="OverallImmigrationShareTable" ref="A1:G6" headerRowCount="1">
-  <autoFilter ref="A1:G6"/>
-  <tableColumns count="7">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="OverallImmigrationShareTable" displayName="OverallImmigrationShareTable" ref="A1:K6" headerRowCount="1">
+  <autoFilter ref="A1:K6"/>
+  <tableColumns count="11">
     <tableColumn id="1" name="Account"/>
     <tableColumn id="2" name="All posts"/>
-    <tableColumn id="3" name="Immigration/enforcement-related posts"/>
-    <tableColumn id="4" name="Immigration share"/>
-    <tableColumn id="5" name="All video posts"/>
-    <tableColumn id="6" name="Immigration/enforcement video posts"/>
-    <tableColumn id="7" name="Immigration share of videos"/>
+    <tableColumn id="3" name="Explicit immigration posts"/>
+    <tableColumn id="4" name="Explicit immigration share"/>
+    <tableColumn id="5" name="Broad immigration/enforcement posts"/>
+    <tableColumn id="6" name="Broad immigration/enforcement share"/>
+    <tableColumn id="7" name="All video posts"/>
+    <tableColumn id="8" name="Explicit immigration video posts"/>
+    <tableColumn id="9" name="Explicit share of videos"/>
+    <tableColumn id="10" name="Broad immigration/enforcement video posts"/>
+    <tableColumn id="11" name="Broad share of videos"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -679,7 +683,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -769,7 +773,7 @@
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>Overall immigration-related posts</t>
+          <t>Explicit immigration-related posts</t>
         </is>
       </c>
       <c r="B7" s="6" t="n">
@@ -785,15 +789,15 @@
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>Unique creative videos</t>
+          <t>Broad immigration/enforcement posts</t>
         </is>
       </c>
       <c r="B8" s="6" t="n">
-        <v>29</v>
+        <v>6063</v>
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>Deduped by media_id where available, otherwise tweet_id.</t>
+          <t>60.6% of all posts in the four target account files.</t>
         </is>
       </c>
       <c r="D8" s="6" t="inlineStr"/>
@@ -801,42 +805,58 @@
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>Latest creative video</t>
-        </is>
-      </c>
-      <c r="B9" s="6" t="inlineStr">
-        <is>
-          <t>2026-05-20T22:22:45.000Z</t>
-        </is>
+          <t>Unique creative videos</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="n">
+        <v>29</v>
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>DHSgov</t>
-        </is>
-      </c>
-      <c r="D9" s="6" t="inlineStr">
-        <is>
-          <t>https://x.com/DHSgov/status/2057225541757903141</t>
-        </is>
-      </c>
+          <t>Deduped by media_id where available, otherwise tweet_id.</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
+          <t>Latest creative video</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-20T22:22:45.000Z</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>DHSgov</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>https://x.com/DHSgov/status/2057225541757903141</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="B10" s="6" t="inlineStr">
+      <c r="B11" s="6" t="inlineStr">
         <is>
           <t>Video-type and slogan/format columns are not mutually exclusive.</t>
         </is>
       </c>
-      <c r="C10" s="6" t="inlineStr">
+      <c r="C11" s="6" t="inlineStr">
         <is>
           <t>A post/video can count in multiple type columns.</t>
         </is>
       </c>
-      <c r="D10" s="6" t="inlineStr"/>
+      <c r="D11" s="6" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -11670,16 +11690,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:K6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
     <col width="11" customWidth="1" min="2" max="2"/>
-    <col width="39" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="17" customWidth="1" min="5" max="5"/>
-    <col width="37" customWidth="1" min="6" max="6"/>
-    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="37" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="17" customWidth="1" min="7" max="7"/>
+    <col width="34" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="43" customWidth="1" min="10" max="10"/>
+    <col width="22" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -11695,27 +11719,47 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Immigration/enforcement-related posts</t>
+          <t>Explicit immigration posts</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Immigration share</t>
+          <t>Explicit immigration share</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>Broad immigration/enforcement posts</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Broad immigration/enforcement share</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
           <t>All video posts</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Immigration/enforcement video posts</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Immigration share of videos</t>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Explicit immigration video posts</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Explicit share of videos</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Broad immigration/enforcement video posts</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Broad share of videos</t>
         </is>
       </c>
     </row>
@@ -11735,13 +11779,25 @@
         <v>0.7653305926687222</v>
       </c>
       <c r="E2" s="6" t="n">
+        <v>2356</v>
+      </c>
+      <c r="F2" s="7" t="n">
+        <v>0.8071257279890374</v>
+      </c>
+      <c r="G2" s="6" t="n">
         <v>790</v>
       </c>
-      <c r="F2" s="6" t="n">
+      <c r="H2" s="6" t="n">
         <v>579</v>
       </c>
-      <c r="G2" s="7" t="n">
+      <c r="I2" s="7" t="n">
         <v>0.7329113924050633</v>
+      </c>
+      <c r="J2" s="6" t="n">
+        <v>626</v>
+      </c>
+      <c r="K2" s="7" t="n">
+        <v>0.7924050632911392</v>
       </c>
     </row>
     <row r="3" ht="30" customHeight="1">
@@ -11760,13 +11816,25 @@
         <v>0.09016393442622951</v>
       </c>
       <c r="E3" s="6" t="n">
+        <v>272</v>
+      </c>
+      <c r="F3" s="7" t="n">
+        <v>0.1013412816691505</v>
+      </c>
+      <c r="G3" s="6" t="n">
         <v>573</v>
       </c>
-      <c r="F3" s="6" t="n">
+      <c r="H3" s="6" t="n">
         <v>55</v>
       </c>
-      <c r="G3" s="7" t="n">
+      <c r="I3" s="7" t="n">
         <v>0.09598603839441536</v>
+      </c>
+      <c r="J3" s="6" t="n">
+        <v>62</v>
+      </c>
+      <c r="K3" s="7" t="n">
+        <v>0.1082024432809773</v>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
@@ -11785,13 +11853,25 @@
         <v>0.8321018062397373</v>
       </c>
       <c r="E4" s="6" t="n">
+        <v>2096</v>
+      </c>
+      <c r="F4" s="7" t="n">
+        <v>0.8604269293924466</v>
+      </c>
+      <c r="G4" s="6" t="n">
         <v>370</v>
       </c>
-      <c r="F4" s="6" t="n">
+      <c r="H4" s="6" t="n">
         <v>322</v>
       </c>
-      <c r="G4" s="7" t="n">
+      <c r="I4" s="7" t="n">
         <v>0.8702702702702703</v>
+      </c>
+      <c r="J4" s="6" t="n">
+        <v>341</v>
+      </c>
+      <c r="K4" s="7" t="n">
+        <v>0.9216216216216216</v>
       </c>
     </row>
     <row r="5" ht="30" customHeight="1">
@@ -11810,13 +11890,25 @@
         <v>0.6610772357723578</v>
       </c>
       <c r="E5" s="6" t="n">
+        <v>1339</v>
+      </c>
+      <c r="F5" s="7" t="n">
+        <v>0.6803861788617886</v>
+      </c>
+      <c r="G5" s="6" t="n">
         <v>205</v>
       </c>
-      <c r="F5" s="6" t="n">
+      <c r="H5" s="6" t="n">
         <v>155</v>
       </c>
-      <c r="G5" s="7" t="n">
+      <c r="I5" s="7" t="n">
         <v>0.7560975609756098</v>
+      </c>
+      <c r="J5" s="6" t="n">
+        <v>162</v>
+      </c>
+      <c r="K5" s="7" t="n">
+        <v>0.7902439024390244</v>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1">
@@ -11835,17 +11927,29 @@
         <v>0.579994004197062</v>
       </c>
       <c r="E6" s="6" t="n">
+        <v>6063</v>
+      </c>
+      <c r="F6" s="7" t="n">
+        <v>0.6058758868791846</v>
+      </c>
+      <c r="G6" s="6" t="n">
         <v>1938</v>
       </c>
-      <c r="F6" s="6" t="n">
+      <c r="H6" s="6" t="n">
         <v>1111</v>
       </c>
-      <c r="G6" s="7" t="n">
+      <c r="I6" s="7" t="n">
         <v>0.5732714138286894</v>
       </c>
+      <c r="J6" s="6" t="n">
+        <v>1191</v>
+      </c>
+      <c r="K6" s="7" t="n">
+        <v>0.6145510835913313</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G6"/>
+  <autoFilter ref="A1:K6"/>
   <conditionalFormatting sqref="B2:B6">
     <cfRule type="dataBar" priority="1">
       <dataBar showValue="1">
@@ -11893,6 +11997,42 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="G2:G6">
     <cfRule type="dataBar" priority="6">
+      <dataBar showValue="1">
+        <cfvo type="num" val="0"/>
+        <cfvo type="max"/>
+        <color rgb="005B9BD5"/>
+      </dataBar>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H2:H6">
+    <cfRule type="dataBar" priority="7">
+      <dataBar showValue="1">
+        <cfvo type="num" val="0"/>
+        <cfvo type="max"/>
+        <color rgb="005B9BD5"/>
+      </dataBar>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I2:I6">
+    <cfRule type="dataBar" priority="8">
+      <dataBar showValue="1">
+        <cfvo type="num" val="0"/>
+        <cfvo type="max"/>
+        <color rgb="005B9BD5"/>
+      </dataBar>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J2:J6">
+    <cfRule type="dataBar" priority="9">
+      <dataBar showValue="1">
+        <cfvo type="num" val="0"/>
+        <cfvo type="max"/>
+        <color rgb="005B9BD5"/>
+      </dataBar>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K2:K6">
+    <cfRule type="dataBar" priority="10">
       <dataBar showValue="1">
         <cfvo type="num" val="0"/>
         <cfvo type="max"/>

</xml_diff>

<commit_message>
Use topic immigration tag in creative workbook
</commit_message>
<xml_diff>
--- a/data/exports/creative-post-video-slogan-stats.xlsx
+++ b/data/exports/creative-post-video-slogan-stats.xlsx
@@ -20,7 +20,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Video Type Summary'!$A$1:$L$6</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Overall Immigration Share'!$A$1:$K$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Overall Immigration Share'!$A$1:$G$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Creative Format Summary'!$A$1:$N$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Tag Overview Videos'!$A$1:$L$105</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Tag Overview All Posts'!$A$1:$L$156</definedName>
@@ -234,20 +234,16 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="OverallImmigrationShareTable" displayName="OverallImmigrationShareTable" ref="A1:K6" headerRowCount="1">
-  <autoFilter ref="A1:K6"/>
-  <tableColumns count="11">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="OverallImmigrationShareTable" displayName="OverallImmigrationShareTable" ref="A1:G6" headerRowCount="1">
+  <autoFilter ref="A1:G6"/>
+  <tableColumns count="7">
     <tableColumn id="1" name="Account"/>
     <tableColumn id="2" name="All posts"/>
-    <tableColumn id="3" name="Explicit immigration posts"/>
-    <tableColumn id="4" name="Explicit immigration share"/>
-    <tableColumn id="5" name="Broad immigration/enforcement posts"/>
-    <tableColumn id="6" name="Broad immigration/enforcement share"/>
-    <tableColumn id="7" name="All video posts"/>
-    <tableColumn id="8" name="Explicit immigration video posts"/>
-    <tableColumn id="9" name="Explicit share of videos"/>
-    <tableColumn id="10" name="Broad immigration/enforcement video posts"/>
-    <tableColumn id="11" name="Broad share of videos"/>
+    <tableColumn id="3" name="topic:immigration posts"/>
+    <tableColumn id="4" name="topic:immigration share"/>
+    <tableColumn id="5" name="All video posts"/>
+    <tableColumn id="6" name="topic:immigration video posts"/>
+    <tableColumn id="7" name="topic:immigration share of videos"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -683,7 +679,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -773,15 +769,15 @@
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>Explicit immigration-related posts</t>
+          <t>topic:immigration posts</t>
         </is>
       </c>
       <c r="B7" s="6" t="n">
-        <v>5804</v>
+        <v>9196</v>
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>58.0% of all posts in the four target account files.</t>
+          <t>91.9% of all posts in the four target account files.</t>
         </is>
       </c>
       <c r="D7" s="6" t="inlineStr"/>
@@ -789,15 +785,15 @@
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>Broad immigration/enforcement posts</t>
+          <t>Unique creative videos</t>
         </is>
       </c>
       <c r="B8" s="6" t="n">
-        <v>6063</v>
+        <v>29</v>
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>60.6% of all posts in the four target account files.</t>
+          <t>Deduped by media_id where available, otherwise tweet_id.</t>
         </is>
       </c>
       <c r="D8" s="6" t="inlineStr"/>
@@ -805,58 +801,42 @@
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>Unique creative videos</t>
-        </is>
-      </c>
-      <c r="B9" s="6" t="n">
-        <v>29</v>
+          <t>Latest creative video</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-20T22:22:45.000Z</t>
+        </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>Deduped by media_id where available, otherwise tweet_id.</t>
-        </is>
-      </c>
-      <c r="D9" s="6" t="inlineStr"/>
+          <t>DHSgov</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>https://x.com/DHSgov/status/2057225541757903141</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>Latest creative video</t>
+          <t>Notes</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>2026-05-20T22:22:45.000Z</t>
+          <t>Video-type and slogan/format columns are not mutually exclusive.</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>DHSgov</t>
-        </is>
-      </c>
-      <c r="D10" s="6" t="inlineStr">
-        <is>
-          <t>https://x.com/DHSgov/status/2057225541757903141</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="5" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
-      <c r="B11" s="6" t="inlineStr">
-        <is>
-          <t>Video-type and slogan/format columns are not mutually exclusive.</t>
-        </is>
-      </c>
-      <c r="C11" s="6" t="inlineStr">
-        <is>
           <t>A post/video can count in multiple type columns.</t>
         </is>
       </c>
-      <c r="D11" s="6" t="inlineStr"/>
+      <c r="D10" s="6" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -11459,10 +11439,10 @@
         <v>0</v>
       </c>
       <c r="K3" s="6" t="n">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="L3" s="6" t="n">
-        <v>438</v>
+        <v>436</v>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
@@ -11579,10 +11559,10 @@
         <v>2</v>
       </c>
       <c r="K6" s="6" t="n">
-        <v>593</v>
+        <v>595</v>
       </c>
       <c r="L6" s="6" t="n">
-        <v>1091</v>
+        <v>1089</v>
       </c>
     </row>
   </sheetData>
@@ -11690,20 +11670,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K6"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
     <col width="11" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="37" customWidth="1" min="5" max="5"/>
-    <col width="24" customWidth="1" min="6" max="6"/>
-    <col width="17" customWidth="1" min="7" max="7"/>
-    <col width="34" customWidth="1" min="8" max="8"/>
-    <col width="22" customWidth="1" min="9" max="9"/>
-    <col width="43" customWidth="1" min="10" max="10"/>
-    <col width="22" customWidth="1" min="11" max="11"/>
+    <col width="25" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="31" customWidth="1" min="6" max="6"/>
+    <col width="28" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -11719,47 +11695,27 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Explicit immigration posts</t>
+          <t>topic:immigration posts</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Explicit immigration share</t>
+          <t>topic:immigration share</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Broad immigration/enforcement posts</t>
+          <t>All video posts</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Broad immigration/enforcement share</t>
+          <t>topic:immigration video posts</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>All video posts</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Explicit immigration video posts</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>Explicit share of videos</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>Broad immigration/enforcement video posts</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>Broad share of videos</t>
+          <t>topic:immigration share of videos</t>
         </is>
       </c>
     </row>
@@ -11773,31 +11729,19 @@
         <v>2919</v>
       </c>
       <c r="C2" s="6" t="n">
-        <v>2234</v>
+        <v>2825</v>
       </c>
       <c r="D2" s="7" t="n">
-        <v>0.7653305926687222</v>
+        <v>0.9677971908187736</v>
       </c>
       <c r="E2" s="6" t="n">
-        <v>2356</v>
-      </c>
-      <c r="F2" s="7" t="n">
-        <v>0.8071257279890374</v>
-      </c>
-      <c r="G2" s="6" t="n">
         <v>790</v>
       </c>
-      <c r="H2" s="6" t="n">
-        <v>579</v>
-      </c>
-      <c r="I2" s="7" t="n">
-        <v>0.7329113924050633</v>
-      </c>
-      <c r="J2" s="6" t="n">
-        <v>626</v>
-      </c>
-      <c r="K2" s="7" t="n">
-        <v>0.7924050632911392</v>
+      <c r="F2" s="6" t="n">
+        <v>756</v>
+      </c>
+      <c r="G2" s="7" t="n">
+        <v>0.9569620253164557</v>
       </c>
     </row>
     <row r="3" ht="30" customHeight="1">
@@ -11810,31 +11754,19 @@
         <v>2684</v>
       </c>
       <c r="C3" s="6" t="n">
-        <v>242</v>
+        <v>1993</v>
       </c>
       <c r="D3" s="7" t="n">
-        <v>0.09016393442622951</v>
+        <v>0.742548435171386</v>
       </c>
       <c r="E3" s="6" t="n">
-        <v>272</v>
-      </c>
-      <c r="F3" s="7" t="n">
-        <v>0.1013412816691505</v>
-      </c>
-      <c r="G3" s="6" t="n">
         <v>573</v>
       </c>
-      <c r="H3" s="6" t="n">
-        <v>55</v>
-      </c>
-      <c r="I3" s="7" t="n">
-        <v>0.09598603839441536</v>
-      </c>
-      <c r="J3" s="6" t="n">
-        <v>62</v>
-      </c>
-      <c r="K3" s="7" t="n">
-        <v>0.1082024432809773</v>
+      <c r="F3" s="6" t="n">
+        <v>410</v>
+      </c>
+      <c r="G3" s="7" t="n">
+        <v>0.7155322862129145</v>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
@@ -11847,31 +11779,19 @@
         <v>2436</v>
       </c>
       <c r="C4" s="6" t="n">
-        <v>2027</v>
+        <v>2424</v>
       </c>
       <c r="D4" s="7" t="n">
-        <v>0.8321018062397373</v>
+        <v>0.9950738916256158</v>
       </c>
       <c r="E4" s="6" t="n">
-        <v>2096</v>
-      </c>
-      <c r="F4" s="7" t="n">
-        <v>0.8604269293924466</v>
-      </c>
-      <c r="G4" s="6" t="n">
         <v>370</v>
       </c>
-      <c r="H4" s="6" t="n">
-        <v>322</v>
-      </c>
-      <c r="I4" s="7" t="n">
-        <v>0.8702702702702703</v>
-      </c>
-      <c r="J4" s="6" t="n">
-        <v>341</v>
-      </c>
-      <c r="K4" s="7" t="n">
-        <v>0.9216216216216216</v>
+      <c r="F4" s="6" t="n">
+        <v>370</v>
+      </c>
+      <c r="G4" s="7" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="5" ht="30" customHeight="1">
@@ -11884,31 +11804,19 @@
         <v>1968</v>
       </c>
       <c r="C5" s="6" t="n">
-        <v>1301</v>
+        <v>1954</v>
       </c>
       <c r="D5" s="7" t="n">
-        <v>0.6610772357723578</v>
+        <v>0.9928861788617886</v>
       </c>
       <c r="E5" s="6" t="n">
-        <v>1339</v>
-      </c>
-      <c r="F5" s="7" t="n">
-        <v>0.6803861788617886</v>
-      </c>
-      <c r="G5" s="6" t="n">
         <v>205</v>
       </c>
-      <c r="H5" s="6" t="n">
-        <v>155</v>
-      </c>
-      <c r="I5" s="7" t="n">
-        <v>0.7560975609756098</v>
-      </c>
-      <c r="J5" s="6" t="n">
-        <v>162</v>
-      </c>
-      <c r="K5" s="7" t="n">
-        <v>0.7902439024390244</v>
+      <c r="F5" s="6" t="n">
+        <v>205</v>
+      </c>
+      <c r="G5" s="7" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1">
@@ -11921,35 +11829,23 @@
         <v>10007</v>
       </c>
       <c r="C6" s="6" t="n">
-        <v>5804</v>
+        <v>9196</v>
       </c>
       <c r="D6" s="7" t="n">
-        <v>0.579994004197062</v>
+        <v>0.9189567302887979</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>6063</v>
-      </c>
-      <c r="F6" s="7" t="n">
-        <v>0.6058758868791846</v>
-      </c>
-      <c r="G6" s="6" t="n">
         <v>1938</v>
       </c>
-      <c r="H6" s="6" t="n">
-        <v>1111</v>
-      </c>
-      <c r="I6" s="7" t="n">
-        <v>0.5732714138286894</v>
-      </c>
-      <c r="J6" s="6" t="n">
-        <v>1191</v>
-      </c>
-      <c r="K6" s="7" t="n">
-        <v>0.6145510835913313</v>
+      <c r="F6" s="6" t="n">
+        <v>1741</v>
+      </c>
+      <c r="G6" s="7" t="n">
+        <v>0.8983488132094943</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K6"/>
+  <autoFilter ref="A1:G6"/>
   <conditionalFormatting sqref="B2:B6">
     <cfRule type="dataBar" priority="1">
       <dataBar showValue="1">
@@ -11997,42 +11893,6 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="G2:G6">
     <cfRule type="dataBar" priority="6">
-      <dataBar showValue="1">
-        <cfvo type="num" val="0"/>
-        <cfvo type="max"/>
-        <color rgb="005B9BD5"/>
-      </dataBar>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H2:H6">
-    <cfRule type="dataBar" priority="7">
-      <dataBar showValue="1">
-        <cfvo type="num" val="0"/>
-        <cfvo type="max"/>
-        <color rgb="005B9BD5"/>
-      </dataBar>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I2:I6">
-    <cfRule type="dataBar" priority="8">
-      <dataBar showValue="1">
-        <cfvo type="num" val="0"/>
-        <cfvo type="max"/>
-        <color rgb="005B9BD5"/>
-      </dataBar>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J2:J6">
-    <cfRule type="dataBar" priority="9">
-      <dataBar showValue="1">
-        <cfvo type="num" val="0"/>
-        <cfvo type="max"/>
-        <color rgb="005B9BD5"/>
-      </dataBar>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="K2:K6">
-    <cfRule type="dataBar" priority="10">
       <dataBar showValue="1">
         <cfvo type="num" val="0"/>
         <cfvo type="max"/>

</xml_diff>